<commit_message>
Integrate Member 2 fixes
</commit_message>
<xml_diff>
--- a/member1_deliverables/Testing_Workbook.xlsx
+++ b/member1_deliverables/Testing_Workbook.xlsx
@@ -59,7 +59,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1644,12 +1644,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">armed=false then true; horizontal velocity=(5,5)</t>
+          <t xml:space="preserve">armed=false then true; distance10m; thrust1; velocity=(5,5,5)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:112; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:201 (GroundContactMCDC_ConditionA_Armed); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1701,12 +1701,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:125; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:217 (GroundContactMCDC_ConditionB_CloseToGround); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:142; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:234 (GroundContactMCDC_ConditionC_LowThrottle); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1785,12 +1785,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:158; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:250 (GroundContactMCDC_ConditionD_HorizontalMovement); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1827,12 +1827,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:174; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:266 (GroundContactMCDC_ConditionE_VerticalMovement); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1854,12 +1854,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">thrust1; armed=false then true</t>
+          <t xml:space="preserve">thrust1; freefall; rotation(5,5,0); stale position; no ground contact; armed=false then true</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1869,12 +1869,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:196; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:288 (MaybeLandedMCDC_ConditionA_Armed); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:209; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:305 (MaybeLandedMCDC_ConditionB_MinThrust); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:225; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:321 (MaybeLandedMCDC_ConditionC_NotFreefall); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="46" ht="72" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_09</t>
+          <t xml:space="preserve">TC_M2_16</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1975,17 +1975,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionE_VerticalEstimate</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">armed; thrust0; no freefall; ground contact; rotation0 then(5,5,0)</t>
+          <t xml:space="preserve">controlled clock20s; G=true after8s; F=false; position exactly1s old then fresh</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -1995,39 +1995,39 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:241; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:337 (MaybeLandedMCDC_ConditionE_VerticalEstimate); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="47" ht="72" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_10</t>
+          <t xml:space="preserve">TC_M2_17</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+          <t xml:space="preserve">MulticopterLandDetector::_get_maybe_landed_state</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionF_GroundContactHysteresis</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no horizontal movement; height flag false; DISARMED; descend true then false</t>
+          <t xml:space="preserve">fresh vertical estimate; G=false; toggle ground contact true then false</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2037,39 +2037,39 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:262; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:361 (MaybeLandedMCDC_ConditionF_GroundContactHysteresis); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="48" ht="72" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_11</t>
+          <t xml:space="preserve">TC_M2_18</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+          <t xml:space="preserve">MulticopterLandDetector::_get_maybe_landed_state</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionG_MinThrust8sHysteresis</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">descending; height flag false; DISARMED; vx0 then5; refresh movement flags</t>
+          <t xml:space="preserve">position exactly1s old; F=false; G=true after8s then false</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2079,39 +2079,39 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:277; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:383 (MaybeLandedMCDC_ConditionG_MinThrust8sHysteresis); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="49" ht="72" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_12</t>
+          <t xml:space="preserve">TC_M2_09</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+          <t xml:space="preserve">MulticopterLandDetector::_get_maybe_landed_state</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">not descending; FLIGHT; height flag true then false</t>
+          <t xml:space="preserve">armed; thrust0; no freefall; ground contact; rotation0 then(5,5,0)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2121,19 +2121,19 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:293; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:405 (MaybeLandedMCDC_ConditionD_NotRotating); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="50" ht="72" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_13</t>
+          <t xml:space="preserve">TC_M2_10</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2143,17 +2143,17 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup</t>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">not descending; height flag false; RAMPUP then DISARMED</t>
+          <t xml:space="preserve">no horizontal movement; height flag false; DISARMED; descend true then false</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision true then false; complete atomic-condition matrix remains unverified</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2163,39 +2163,39 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:308; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:426 (GroundEffectMCDC_ConditionA_InDescend); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="51" ht="72" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC_M2_14</t>
+          <t xml:space="preserve">TC_M2_11</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector::_get_freefall_state</t>
+          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freefall_AccelThresholdBoundary</t>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acceleration(1,0,1) then(0,0,9.81)</t>
+          <t xml:space="preserve">descending remains true; height flag false; DISARMED; cached horizontal movement false then true; all other D3 operands fixed</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freefall true then false</t>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2205,59 +2205,227 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:327; logs/member2_execution.xml</t>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:441 (GroundEffectMCDC_ConditionB_NoHorizontalMovement); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
     <row r="52" ht="72" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">TC_M2_12</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">not descending; FLIGHT; height flag true then false</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:456 (GroundEffectMCDC_ConditionC_BelowGndHeight); logs/member2_execution.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="72" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC_M2_19</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionD_TakeoffStateFlight</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">not descending; cached horizontal movement true; below height; FLIGHT then DISARMED</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:471 (GroundEffectMCDC_ConditionD_TakeoffStateFlight); logs/member2_execution.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC_M2_13</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector::_get_ground_effect_state</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">not descending; height flag false; RAMPUP then DISARMED</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision true then false; assert all controlled D1-D3 operand values and record runtime vectors</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:490 (GroundEffectMCDC_ConditionE_TakeoffRampup); logs/member2_execution.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC_M2_14</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector::_get_freefall_state</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freefall_AccelThresholdBoundary</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Acceleration(1,0,1) then(0,0,9.81)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freefall true then false</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:509 (Freefall_AccelThresholdBoundary); logs/member2_execution.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="72" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">TC_M2_15</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">MulticopterLandDetector::_get_landed_state</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Landed_StateTransitions</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Disarmed; armed+maybe_landed true; armed+maybe_landed false</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Landed true, true, false</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PASS</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Imported Member 2 decision tests; see integration_notes.md</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:338; logs/member2_execution.xml</t>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3 return-decision pairs verified against runtime vectors; broader governing guards pending</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/modules/land_detector/LandDetectorTest.cpp:520 (Landed_StateTransitions); logs/member2_execution.xml</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H56"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -2265,7 +2433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2364,12 +2532,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionA_Armed (Line 104)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionA_Armed (TP_D1_A1)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionA_Armed (Line 110)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionA_Armed (TP_D1_A2)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2458,12 +2626,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionB_CloseToGround (Line 123)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionB_CloseToGround (TP_D1_B1)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2505,12 +2673,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionB_CloseToGround (Line 127)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionB_CloseToGround (TP_D1_B2)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2547,17 +2715,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition C (ground_contact)</t>
+          <t xml:space="preserve">Condition C (ground_contact / low throttle)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionC_LowThrottle (Line 140)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionC_LowThrottle (TP_D1_C1)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2594,17 +2762,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition C (ground_contact)</t>
+          <t xml:space="preserve">Condition C (ground_contact / low throttle)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionC_LowThrottle (Line 144)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionC_LowThrottle (TP_D1_C2)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2646,12 +2814,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionD_HorizontalMovement (Line 157)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionD_HorizontalMovement (TP_D1_D1)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2693,12 +2861,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionD_HorizontalMovement (Line 161)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionD_HorizontalMovement (TP_D1_D2)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2740,12 +2908,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionE_VerticalMovement (Line 174)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionE_VerticalMovement (TP_D1_E1)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2787,12 +2955,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundContactMCDC_ConditionE_VerticalMovement (Line 178)</t>
+          <t xml:space="preserve">GroundContactMCDC_ConditionE_VerticalMovement (TP_D1_E2)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2834,12 +3002,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionA_Armed (Line 191)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionA_Armed (TP_D2_A1)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2881,12 +3049,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionA_Armed (Line 196)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionA_Armed (TP_D2_A2)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2928,12 +3096,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionB_MinThrust (Line 209)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionB_MinThrust (TP_D2_B1)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -2975,12 +3143,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionB_MinThrust (Line 213)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionB_MinThrust (TP_D2_B2)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3022,12 +3190,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionC_NotFreefall (Line 225)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionC_NotFreefall (TP_D2_C1)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3069,12 +3237,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionC_NotFreefall (Line 229)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionC_NotFreefall (TP_D2_C2)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3284,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating (Line 241)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating (TP_D2_D1)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3163,34 +3331,34 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating (Line 245)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionD_NotRotating (TP_D2_D2)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="72" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T T F F F]</t>
+          <t xml:space="preserve">[F T T T F F T]</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3200,44 +3368,44 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_A1 TP_D3_A2)</t>
+          <t xml:space="preserve">Pair (TP_D2_E1 TP_D2_E2)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition A (in_descend)</t>
+          <t xml:space="preserve">Condition E (vertical_estimate = local_pos_updated AND v_z_valid)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend (Line 262)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionE_VerticalEstimate (TP_D2_E1)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="72" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[F T F F F]</t>
+          <t xml:space="preserve">[F T T T T F T]</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3247,44 +3415,44 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_A1 TP_D3_A2)</t>
+          <t xml:space="preserve">Pair (TP_D2_E1 TP_D2_E2)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition A (in_descend)</t>
+          <t xml:space="preserve">Condition E (vertical_estimate = local_pos_updated AND v_z_valid)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend (Line 266)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionE_VerticalEstimate (TP_D2_E2)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="72" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T T F F F]</t>
+          <t xml:space="preserve">[F T T T T T F]</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -3294,44 +3462,44 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_B1 TP_D3_B2)</t>
+          <t xml:space="preserve">Pair (TP_D2_F1 TP_D2_F2)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition B (!horizontal_mov)</t>
+          <t xml:space="preserve">Condition F (_ground_contact_hysteresis)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement (Line 277)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionF_GroundContactHysteresis (TP_D2_F1)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[T F F F F]</t>
+          <t xml:space="preserve">[F T T T T F F]</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3341,44 +3509,44 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_B1 TP_D3_B2)</t>
+          <t xml:space="preserve">Pair (TP_D2_F1 TP_D2_F2)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition B (!horizontal_mov)</t>
+          <t xml:space="preserve">Condition F (_ground_contact_hysteresis)</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement (Line 288)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionF_GroundContactHysteresis (TP_D2_F2)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="72" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[F F T T F]</t>
+          <t xml:space="preserve">[F T T T F F T]</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3388,44 +3556,44 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_C1 TP_D3_C2)</t>
+          <t xml:space="preserve">Pair (TP_D2_G1 TP_D2_G2)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition C (below_gnd_effect)</t>
+          <t xml:space="preserve">Condition G (_minimum_thrust_8s_hysteresis)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight (Line 293)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionG_MinThrust8sHysteresis (TP_D2_G1)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="72" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:287</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+          <t xml:space="preserve">A OR (B AND C AND D AND ((E AND F) OR (NOT E AND G)))</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[F F F T F]</t>
+          <t xml:space="preserve">[F T T T F F F]</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -3435,22 +3603,22 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_C1 TP_D3_C2)</t>
+          <t xml:space="preserve">Pair (TP_D2_G1 TP_D2_G2)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition C (below_gnd_effect)</t>
+          <t xml:space="preserve">Condition G (_minimum_thrust_8s_hysteresis)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight (Line 297)</t>
+          <t xml:space="preserve">MaybeLandedMCDC_ConditionG_MinThrust8sHysteresis (TP_D2_G2)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3640,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[F F F F T]</t>
+          <t xml:space="preserve">[T T F F F]</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3482,22 +3650,22 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pair (TP_D3_E1 TP_D3_E2)</t>
+          <t xml:space="preserve">Pair (TP_D3_A1 TP_D3_A2)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition E (takeoff_rampup)</t>
+          <t xml:space="preserve">Condition A (in_descend)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup (Line 308)</t>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend (TP_D3_A1)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
@@ -3519,37 +3687,413 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">[F T F F F]</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_A1 TP_D3_A2)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition A (in_descend)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionA_InDescend (TP_D3_A2)</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="72" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[T T F F F]</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_B1 TP_D3_B2)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition B (!horizontal_mov)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement (TP_D3_B1)</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[T F F F F]</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_B1 TP_D3_B2)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition B (!horizontal_mov)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionB_NoHorizontalMovement (TP_D3_B2)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[F F T T F]</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_C1 TP_D3_C2)</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition C (below_gnd_effect)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight (TP_D3_C1)</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[F F F T F]</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_C1 TP_D3_C2)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition C (below_gnd_effect)</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionC_BelowGndHeight (TP_D3_C2)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[F F T T F]</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_D1 TP_D3_D2)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition D (takeoff_state == TAKEOFF_STATE_FLIGHT)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionD_TakeoffStateFlight (TP_D3_D1)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[F F T F F]</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_D1 TP_D3_D2)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition D (takeoff_state == TAKEOFF_STATE_FLIGHT)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionD_TakeoffStateFlight (TP_D3_D2)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[F F F F T]</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pair (TP_D3_E1 TP_D3_E2)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition E (takeoff_state == TAKEOFF_STATE_RAMPUP)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup (TP_D3_E1)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D3</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MulticopterLandDetector.cpp:300</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(A AND B) OR (C AND D) OR E</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">[F F F F F]</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">False</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Pair (TP_D3_E1 TP_D3_E2)</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Condition E (takeoff_rampup)</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup (Line 312)</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Imported from Member 2; execution rechecked; matrix not certified. Missing D2 E/F/G and D3 D pairs; see integration_notes.md.</t>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condition E (takeoff_state == TAKEOFF_STATE_RAMPUP)</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GroundEffectMCDC_ConditionE_TakeoffRampup (TP_D3_E2)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1-D3: runtime operands/outcomes checked; 17 single-condition pairs validated. Masks follow source short-circuit rules. Other governing guards remain to be analyzed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I27"/>
+  <autoFilter ref="A1:I35"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>